<commit_message>
init comit CBA analysis tornado & whirpool
</commit_message>
<xml_diff>
--- a/ssp_modeling/cost-benefits/cb_config_files/cb_config_params.xlsx
+++ b/ssp_modeling/cost-benefits/cb_config_files/cb_config_params.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10302"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10315"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fabianfuentes/git/ssp_libya/ssp_modeling/cost-benefits/cb_config_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{774E7CAE-8D20-5440-B586-440310A79CCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DFB0F81-4B49-3C40-BA96-CCBA4A139C98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-51200" yWindow="-7160" windowWidth="25600" windowHeight="28200" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-39500" yWindow="-7160" windowWidth="31780" windowHeight="28200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="tx_table" sheetId="1" r:id="rId1"/>
@@ -6710,7 +6710,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:E213"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
@@ -6757,7 +6756,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="3" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>46</v>
       </c>
@@ -6774,7 +6773,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="4" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>47</v>
       </c>
@@ -6791,7 +6790,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="5" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>48</v>
       </c>
@@ -6808,7 +6807,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="6" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>49</v>
       </c>
@@ -6825,7 +6824,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="7" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>50</v>
       </c>
@@ -6842,7 +6841,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="8" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>51</v>
       </c>
@@ -6859,7 +6858,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="9" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>52</v>
       </c>
@@ -6876,7 +6875,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="10" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>53</v>
       </c>
@@ -6893,7 +6892,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="11" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>54</v>
       </c>
@@ -6910,7 +6909,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="12" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>55</v>
       </c>
@@ -6927,7 +6926,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="13" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>56</v>
       </c>
@@ -6944,7 +6943,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="14" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>57</v>
       </c>
@@ -6961,7 +6960,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="15" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>58</v>
       </c>
@@ -6978,7 +6977,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="16" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>200</v>
       </c>
@@ -6995,7 +6994,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="17" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>198</v>
       </c>
@@ -7012,7 +7011,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="18" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>197</v>
       </c>
@@ -7063,7 +7062,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="21" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>76</v>
       </c>
@@ -7080,7 +7079,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="22" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>61</v>
       </c>
@@ -7097,7 +7096,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="23" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>195</v>
       </c>
@@ -7114,7 +7113,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="24" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>116</v>
       </c>
@@ -7131,7 +7130,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="25" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>117</v>
       </c>
@@ -7148,7 +7147,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="26" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>118</v>
       </c>
@@ -7165,7 +7164,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="27" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>119</v>
       </c>
@@ -7182,7 +7181,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="28" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>120</v>
       </c>
@@ -7199,7 +7198,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="29" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>121</v>
       </c>
@@ -7216,7 +7215,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="30" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>122</v>
       </c>
@@ -7233,7 +7232,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="31" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>123</v>
       </c>
@@ -7250,7 +7249,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="32" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>124</v>
       </c>
@@ -7267,7 +7266,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="33" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>125</v>
       </c>
@@ -7284,7 +7283,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="34" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>126</v>
       </c>
@@ -7301,7 +7300,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="35" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>127</v>
       </c>
@@ -7318,7 +7317,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="36" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>128</v>
       </c>
@@ -7335,7 +7334,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="37" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>129</v>
       </c>
@@ -7352,7 +7351,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="38" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>130</v>
       </c>
@@ -7369,7 +7368,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="39" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>131</v>
       </c>
@@ -7386,7 +7385,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="40" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>132</v>
       </c>
@@ -7403,7 +7402,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="41" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>133</v>
       </c>
@@ -7420,7 +7419,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="42" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>134</v>
       </c>
@@ -7437,7 +7436,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="43" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>135</v>
       </c>
@@ -7454,7 +7453,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="44" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>136</v>
       </c>
@@ -7471,7 +7470,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="45" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>137</v>
       </c>
@@ -7488,7 +7487,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="46" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>138</v>
       </c>
@@ -7505,7 +7504,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="47" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>139</v>
       </c>
@@ -7522,7 +7521,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="48" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>140</v>
       </c>
@@ -7539,7 +7538,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="49" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>141</v>
       </c>
@@ -7556,7 +7555,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="50" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>142</v>
       </c>
@@ -7573,7 +7572,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="51" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>143</v>
       </c>
@@ -7590,7 +7589,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="52" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>144</v>
       </c>
@@ -7607,7 +7606,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="53" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>145</v>
       </c>
@@ -7624,7 +7623,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="54" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>146</v>
       </c>
@@ -7641,7 +7640,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="55" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>147</v>
       </c>
@@ -7658,7 +7657,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="56" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>148</v>
       </c>
@@ -7675,7 +7674,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="57" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>149</v>
       </c>
@@ -7692,7 +7691,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="58" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>150</v>
       </c>
@@ -7709,7 +7708,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="59" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>151</v>
       </c>
@@ -7726,7 +7725,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="60" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>152</v>
       </c>
@@ -7743,7 +7742,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="61" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>153</v>
       </c>
@@ -7760,7 +7759,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="62" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>154</v>
       </c>
@@ -7777,7 +7776,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="63" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>155</v>
       </c>
@@ -7794,7 +7793,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="64" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>156</v>
       </c>
@@ -7811,7 +7810,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="65" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>157</v>
       </c>
@@ -7828,7 +7827,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="66" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>158</v>
       </c>
@@ -7845,7 +7844,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="67" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>159</v>
       </c>
@@ -7862,7 +7861,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="68" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>160</v>
       </c>
@@ -7879,7 +7878,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="69" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>161</v>
       </c>
@@ -7896,7 +7895,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="70" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>162</v>
       </c>
@@ -7913,7 +7912,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="71" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>106</v>
       </c>
@@ -7930,7 +7929,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="72" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>87</v>
       </c>
@@ -7947,7 +7946,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="73" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>85</v>
       </c>
@@ -7964,7 +7963,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="74" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>86</v>
       </c>
@@ -7981,7 +7980,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="75" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>64</v>
       </c>
@@ -7998,7 +7997,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="76" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>12</v>
       </c>
@@ -8032,7 +8031,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="78" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>13</v>
       </c>
@@ -8049,7 +8048,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="79" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>185</v>
       </c>
@@ -8066,7 +8065,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="80" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>191</v>
       </c>
@@ -8083,7 +8082,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="81" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>192</v>
       </c>
@@ -8100,7 +8099,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="82" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>102</v>
       </c>
@@ -8117,7 +8116,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="83" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>103</v>
       </c>
@@ -8134,7 +8133,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="84" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>104</v>
       </c>
@@ -8151,7 +8150,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="85" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>100</v>
       </c>
@@ -8168,7 +8167,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="86" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
         <v>101</v>
       </c>
@@ -8185,7 +8184,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="87" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>105</v>
       </c>
@@ -8202,7 +8201,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="88" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>77</v>
       </c>
@@ -8219,7 +8218,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="89" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>62</v>
       </c>
@@ -8236,7 +8235,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="90" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
         <v>169</v>
       </c>
@@ -8253,7 +8252,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="91" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
         <v>167</v>
       </c>
@@ -8270,7 +8269,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="92" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
         <v>165</v>
       </c>
@@ -8287,7 +8286,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="93" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
         <v>163</v>
       </c>
@@ -8355,7 +8354,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="97" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
         <v>66</v>
       </c>
@@ -8372,7 +8371,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="98" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
         <v>74</v>
       </c>
@@ -8389,7 +8388,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="99" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
         <v>75</v>
       </c>
@@ -8406,7 +8405,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="100" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
         <v>188</v>
       </c>
@@ -8423,7 +8422,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="101" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
         <v>187</v>
       </c>
@@ -8440,7 +8439,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="102" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
         <v>190</v>
       </c>
@@ -8457,7 +8456,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="103" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
         <v>189</v>
       </c>
@@ -8474,7 +8473,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="104" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
         <v>186</v>
       </c>
@@ -8491,7 +8490,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="105" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A105" s="5" t="s">
         <v>2037</v>
       </c>
@@ -8508,7 +8507,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="106" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
         <v>207</v>
       </c>
@@ -8525,7 +8524,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="107" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
         <v>18</v>
       </c>
@@ -8542,7 +8541,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="108" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
         <v>19</v>
       </c>
@@ -8559,7 +8558,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="109" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
         <v>206</v>
       </c>
@@ -8576,7 +8575,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="110" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
         <v>204</v>
       </c>
@@ -8593,7 +8592,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="111" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
         <v>205</v>
       </c>
@@ -8610,7 +8609,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="112" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
         <v>115</v>
       </c>
@@ -8627,7 +8626,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="113" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A113" s="6" t="s">
         <v>2044</v>
       </c>
@@ -8641,7 +8640,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="114" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A114" s="5" t="s">
         <v>2038</v>
       </c>
@@ -8658,7 +8657,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="115" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A115" s="5" t="s">
         <v>2042</v>
       </c>
@@ -8675,7 +8674,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="116" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A116" s="5" t="s">
         <v>2040</v>
       </c>
@@ -8692,7 +8691,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="117" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
         <v>37</v>
       </c>
@@ -8709,7 +8708,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="118" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
         <v>38</v>
       </c>
@@ -8726,7 +8725,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="119" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
         <v>39</v>
       </c>
@@ -8743,7 +8742,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="120" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
         <v>40</v>
       </c>
@@ -8760,7 +8759,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="121" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
         <v>41</v>
       </c>
@@ -8777,7 +8776,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="122" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
         <v>42</v>
       </c>
@@ -8794,7 +8793,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="123" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
         <v>43</v>
       </c>
@@ -8811,7 +8810,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="124" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A124" t="s">
         <v>44</v>
       </c>
@@ -8828,7 +8827,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="125" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A125" t="s">
         <v>45</v>
       </c>
@@ -8845,7 +8844,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="126" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A126" t="s">
         <v>196</v>
       </c>
@@ -8862,7 +8861,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="127" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A127" t="s">
         <v>201</v>
       </c>
@@ -8896,7 +8895,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="129" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A129" t="s">
         <v>202</v>
       </c>
@@ -8913,7 +8912,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="130" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A130" t="s">
         <v>78</v>
       </c>
@@ -8930,7 +8929,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="131" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A131" t="s">
         <v>63</v>
       </c>
@@ -8947,7 +8946,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="132" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A132" t="s">
         <v>181</v>
       </c>
@@ -8964,7 +8963,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="133" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A133" t="s">
         <v>184</v>
       </c>
@@ -8981,7 +8980,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="134" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A134" t="s">
         <v>182</v>
       </c>
@@ -9015,7 +9014,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="136" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A136" t="s">
         <v>99</v>
       </c>
@@ -9032,7 +9031,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="137" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A137" t="s">
         <v>98</v>
       </c>
@@ -9049,7 +9048,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="138" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A138" t="s">
         <v>17</v>
       </c>
@@ -9066,7 +9065,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="139" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A139" t="s">
         <v>15</v>
       </c>
@@ -9083,7 +9082,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="140" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A140" t="s">
         <v>16</v>
       </c>
@@ -9100,7 +9099,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="141" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A141" t="s">
         <v>90</v>
       </c>
@@ -9117,7 +9116,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="142" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A142" t="s">
         <v>88</v>
       </c>
@@ -9134,7 +9133,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="143" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A143" t="s">
         <v>91</v>
       </c>
@@ -9151,7 +9150,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="144" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A144" t="s">
         <v>89</v>
       </c>
@@ -9168,7 +9167,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="145" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A145" t="s">
         <v>109</v>
       </c>
@@ -9185,7 +9184,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="146" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A146" t="s">
         <v>107</v>
       </c>
@@ -9202,7 +9201,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="147" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A147" t="s">
         <v>110</v>
       </c>
@@ -9219,7 +9218,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="148" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A148" t="s">
         <v>108</v>
       </c>
@@ -9236,7 +9235,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="149" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A149" t="s">
         <v>79</v>
       </c>
@@ -9253,7 +9252,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="150" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A150" t="s">
         <v>65</v>
       </c>
@@ -9270,7 +9269,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="151" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A151" t="s">
         <v>20</v>
       </c>
@@ -9287,7 +9286,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="152" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A152" t="s">
         <v>21</v>
       </c>
@@ -9304,7 +9303,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="153" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A153" t="s">
         <v>22</v>
       </c>
@@ -9321,7 +9320,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="154" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A154" t="s">
         <v>23</v>
       </c>
@@ -9338,7 +9337,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="155" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A155" t="s">
         <v>67</v>
       </c>
@@ -9355,7 +9354,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="156" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A156" t="s">
         <v>68</v>
       </c>
@@ -9372,7 +9371,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="157" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A157" t="s">
         <v>69</v>
       </c>
@@ -9389,7 +9388,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="158" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A158" t="s">
         <v>70</v>
       </c>
@@ -9406,7 +9405,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="159" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A159" t="s">
         <v>71</v>
       </c>
@@ -9423,7 +9422,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="160" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A160" t="s">
         <v>72</v>
       </c>
@@ -9440,7 +9439,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="161" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A161" t="s">
         <v>180</v>
       </c>
@@ -9457,7 +9456,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="162" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A162" t="s">
         <v>178</v>
       </c>
@@ -9474,7 +9473,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="163" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="163" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A163" t="s">
         <v>179</v>
       </c>
@@ -9491,7 +9490,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="164" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A164" t="s">
         <v>177</v>
       </c>
@@ -9508,7 +9507,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="165" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="165" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A165" t="s">
         <v>175</v>
       </c>
@@ -9525,7 +9524,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="166" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A166" t="s">
         <v>170</v>
       </c>
@@ -9542,7 +9541,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="167" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="167" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A167" t="s">
         <v>172</v>
       </c>
@@ -9559,7 +9558,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="168" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="168" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A168" t="s">
         <v>174</v>
       </c>
@@ -9627,7 +9626,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="172" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="172" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A172" t="s">
         <v>60</v>
       </c>
@@ -9644,7 +9643,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="173" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="173" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A173" t="s">
         <v>59</v>
       </c>
@@ -9661,7 +9660,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="174" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="174" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A174" t="s">
         <v>32</v>
       </c>
@@ -9678,7 +9677,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="175" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="175" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A175" t="s">
         <v>33</v>
       </c>
@@ -9695,7 +9694,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="176" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="176" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A176" t="s">
         <v>34</v>
       </c>
@@ -9712,7 +9711,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="177" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="177" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A177" t="s">
         <v>30</v>
       </c>
@@ -9729,7 +9728,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="178" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="178" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A178" t="s">
         <v>31</v>
       </c>
@@ -9746,7 +9745,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="179" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="179" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A179" t="s">
         <v>35</v>
       </c>
@@ -9763,7 +9762,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="180" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="180" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A180" t="s">
         <v>114</v>
       </c>
@@ -9780,7 +9779,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="181" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="181" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A181" t="s">
         <v>113</v>
       </c>
@@ -9797,7 +9796,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="182" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="182" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A182" t="s">
         <v>112</v>
       </c>
@@ -9814,7 +9813,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="183" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="183" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A183" t="s">
         <v>111</v>
       </c>
@@ -9831,7 +9830,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="184" spans="1:5" s="5" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
+    <row r="184" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A184" t="s">
         <v>36</v>
       </c>
@@ -9848,7 +9847,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="185" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="185" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A185" t="s">
         <v>6</v>
       </c>
@@ -9865,7 +9864,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="186" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="186" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A186" t="s">
         <v>9</v>
       </c>
@@ -9882,7 +9881,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="187" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="187" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A187" t="s">
         <v>11</v>
       </c>
@@ -9899,7 +9898,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="188" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="188" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A188" t="s">
         <v>7</v>
       </c>
@@ -9916,7 +9915,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="189" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="189" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A189" t="s">
         <v>10</v>
       </c>
@@ -9933,7 +9932,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="190" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="190" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A190" t="s">
         <v>5</v>
       </c>
@@ -9950,7 +9949,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="191" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="191" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A191" t="s">
         <v>8</v>
       </c>
@@ -9984,7 +9983,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="193" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="193" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A193" t="s">
         <v>73</v>
       </c>
@@ -10001,7 +10000,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="194" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="194" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A194" t="s">
         <v>83</v>
       </c>
@@ -10018,7 +10017,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="195" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="195" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A195" t="s">
         <v>84</v>
       </c>
@@ -10035,7 +10034,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="196" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="196" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A196" s="6" t="s">
         <v>2047</v>
       </c>
@@ -10049,7 +10048,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="197" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="197" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A197" t="s">
         <v>193</v>
       </c>
@@ -10066,7 +10065,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="198" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="198" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A198" t="s">
         <v>92</v>
       </c>
@@ -10083,7 +10082,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="199" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="199" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A199" t="s">
         <v>93</v>
       </c>
@@ -10100,7 +10099,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="200" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="200" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A200" t="s">
         <v>94</v>
       </c>
@@ -10117,7 +10116,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="201" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="201" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A201" t="s">
         <v>95</v>
       </c>
@@ -10134,7 +10133,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="202" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="202" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A202" t="s">
         <v>96</v>
       </c>
@@ -10151,7 +10150,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="203" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="203" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A203" t="s">
         <v>97</v>
       </c>
@@ -10168,7 +10167,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="204" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="204" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A204" t="s">
         <v>24</v>
       </c>
@@ -10185,7 +10184,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="205" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="205" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A205" t="s">
         <v>25</v>
       </c>
@@ -10202,7 +10201,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="206" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="206" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A206" t="s">
         <v>26</v>
       </c>
@@ -10219,7 +10218,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="207" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="207" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A207" t="s">
         <v>27</v>
       </c>
@@ -10236,7 +10235,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="208" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="208" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A208" t="s">
         <v>28</v>
       </c>
@@ -10253,7 +10252,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="209" spans="1:5" s="5" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
+    <row r="209" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A209" t="s">
         <v>29</v>
       </c>
@@ -10270,7 +10269,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="210" spans="1:5" s="5" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
+    <row r="210" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A210" t="s">
         <v>81</v>
       </c>
@@ -10287,7 +10286,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="211" spans="1:5" s="5" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
+    <row r="211" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A211" t="s">
         <v>80</v>
       </c>
@@ -10304,7 +10303,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="212" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="212" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A212" t="s">
         <v>82</v>
       </c>
@@ -10321,7 +10320,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="213" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="213" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A213" t="s">
         <v>14</v>
       </c>
@@ -10339,28 +10338,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E213" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="cb:agrc:consumer_savings:cons_ag_land_value:X"/>
-        <filter val="cb:agrc:technical_savings:cons_ag:X"/>
-        <filter val="cb:agrc:technical_savings:producer_food_waste:X"/>
-        <filter val="cb:entc:technical_savings:electricity:opex"/>
-        <filter val="cb:inen:technical_savings:fuel_switch:all"/>
-        <filter val="cb:inen:technical_savings:fuel_switch:hi_heat"/>
-        <filter val="cb:inen:technical_savings:fuel_switch:lo_heat"/>
-        <filter val="cb:pflo:consumer_savings:better_diets:X"/>
-        <filter val="cb:scoe:technical_savings:fuel_switch:heat_pumps"/>
-        <filter val="cb:trns:technical_savings:electrification:hdv_vehicles"/>
-        <filter val="cb:trns:technical_savings:electrification:LDV"/>
-        <filter val="cb:trns:technical_savings:electrification:rail"/>
-        <filter val="cb:waso:consumer_savings:consumer_food_waste:X"/>
-      </filters>
-    </filterColumn>
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E213">
-      <sortCondition ref="A1:A213"/>
-    </sortState>
-  </autoFilter>
+  <autoFilter ref="A1:E213" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <hyperlinks>
     <hyperlink ref="C212" r:id="rId1" location=":~:text=Using%20the%20World%20Bank%20numbers,case%20of%20U.S.%20LMOP%20landfills." xr:uid="{00000000-0004-0000-0000-000000000000}"/>
   </hyperlinks>

</xml_diff>